<commit_message>
Drop the one function Numbers cannot evaluate
The two contested-share columns guarded their division with IF(N(x)=0,...).
Numbers has no N(), so it flagged all 81 of those cells as unsupported
formulas on import. IFERROR(a/b,"") does the same job -- a blank or zero
denominator raises #DIV/0! and is caught -- and every one of Excel,
Numbers, Google Sheets and LibreOffice evaluates it.

The workbook is now down to three functions, IFERROR, SUM and EXP, and the
builder refuses to save a formula using anything outside a list all four
apps support, so this cannot come back silently. All 93 formulas
hand-evaluated against the page's own numbers; the file's XML parses
clean in every part.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CyJT87Xw81b5gvhLUekjFd
</commit_message>
<xml_diff>
--- a/docs/plan-2027.xlsx
+++ b/docs/plan-2027.xlsx
@@ -649,6 +649,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -773,6 +774,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
@@ -864,6 +866,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
@@ -907,6 +910,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
@@ -1071,7 +1075,7 @@
       <c r="L2" s="15" t="n"/>
       <c r="M2" s="15" t="n"/>
       <c r="N2" s="16">
-        <f>IF(N(L2)=0,"",M2/L2)</f>
+        <f>IFERROR(M2/L2,"")</f>
         <v/>
       </c>
       <c r="O2" s="12" t="inlineStr"/>
@@ -1132,7 +1136,7 @@
         <v>4</v>
       </c>
       <c r="N3" s="16">
-        <f>IF(N(L3)=0,"",M3/L3)</f>
+        <f>IFERROR(M3/L3,"")</f>
         <v/>
       </c>
       <c r="O3" s="12" t="inlineStr"/>
@@ -1197,7 +1201,7 @@
         <v>8.25</v>
       </c>
       <c r="N4" s="16">
-        <f>IF(N(L4)=0,"",M4/L4)</f>
+        <f>IFERROR(M4/L4,"")</f>
         <v/>
       </c>
       <c r="O4" s="12" t="inlineStr"/>
@@ -1258,7 +1262,7 @@
         <v>11</v>
       </c>
       <c r="N5" s="16">
-        <f>IF(N(L5)=0,"",M5/L5)</f>
+        <f>IFERROR(M5/L5,"")</f>
         <v/>
       </c>
       <c r="O5" s="12" t="inlineStr"/>
@@ -1323,7 +1327,7 @@
         <v>9.5</v>
       </c>
       <c r="N6" s="16">
-        <f>IF(N(L6)=0,"",M6/L6)</f>
+        <f>IFERROR(M6/L6,"")</f>
         <v/>
       </c>
       <c r="O6" s="12" t="inlineStr"/>
@@ -1380,7 +1384,7 @@
       <c r="L7" s="15" t="n"/>
       <c r="M7" s="15" t="n"/>
       <c r="N7" s="16">
-        <f>IF(N(L7)=0,"",M7/L7)</f>
+        <f>IFERROR(M7/L7,"")</f>
         <v/>
       </c>
       <c r="O7" s="12" t="inlineStr">
@@ -1449,7 +1453,7 @@
         <v>11</v>
       </c>
       <c r="N8" s="16">
-        <f>IF(N(L8)=0,"",M8/L8)</f>
+        <f>IFERROR(M8/L8,"")</f>
         <v/>
       </c>
       <c r="O8" s="12" t="inlineStr">
@@ -1506,7 +1510,7 @@
       <c r="L9" s="15" t="n"/>
       <c r="M9" s="15" t="n"/>
       <c r="N9" s="16">
-        <f>IF(N(L9)=0,"",M9/L9)</f>
+        <f>IFERROR(M9/L9,"")</f>
         <v/>
       </c>
       <c r="O9" s="12" t="inlineStr"/>
@@ -1567,7 +1571,7 @@
         <v>3.25</v>
       </c>
       <c r="N10" s="16">
-        <f>IF(N(L10)=0,"",M10/L10)</f>
+        <f>IFERROR(M10/L10,"")</f>
         <v/>
       </c>
       <c r="O10" s="12" t="inlineStr"/>
@@ -1632,7 +1636,7 @@
         <v>10.5</v>
       </c>
       <c r="N11" s="16">
-        <f>IF(N(L11)=0,"",M11/L11)</f>
+        <f>IFERROR(M11/L11,"")</f>
         <v/>
       </c>
       <c r="O11" s="12" t="inlineStr"/>
@@ -1693,7 +1697,7 @@
         <v>8</v>
       </c>
       <c r="N12" s="16">
-        <f>IF(N(L12)=0,"",M12/L12)</f>
+        <f>IFERROR(M12/L12,"")</f>
         <v/>
       </c>
       <c r="O12" s="12" t="inlineStr">
@@ -1752,7 +1756,7 @@
       <c r="L13" s="15" t="n"/>
       <c r="M13" s="15" t="n"/>
       <c r="N13" s="16">
-        <f>IF(N(L13)=0,"",M13/L13)</f>
+        <f>IFERROR(M13/L13,"")</f>
         <v/>
       </c>
       <c r="O13" s="12" t="inlineStr">
@@ -1817,7 +1821,7 @@
         <v>5.933333333333334</v>
       </c>
       <c r="N14" s="16">
-        <f>IF(N(L14)=0,"",M14/L14)</f>
+        <f>IFERROR(M14/L14,"")</f>
         <v/>
       </c>
       <c r="O14" s="12" t="inlineStr">
@@ -1882,7 +1886,7 @@
         <v>3.047619047619047</v>
       </c>
       <c r="N15" s="16">
-        <f>IF(N(L15)=0,"",M15/L15)</f>
+        <f>IFERROR(M15/L15,"")</f>
         <v/>
       </c>
       <c r="O15" s="12" t="inlineStr">
@@ -1947,7 +1951,7 @@
         <v>0.75</v>
       </c>
       <c r="N16" s="16">
-        <f>IF(N(L16)=0,"",M16/L16)</f>
+        <f>IFERROR(M16/L16,"")</f>
         <v/>
       </c>
       <c r="O16" s="12" t="inlineStr"/>
@@ -2004,7 +2008,7 @@
       <c r="L17" s="15" t="n"/>
       <c r="M17" s="15" t="n"/>
       <c r="N17" s="16">
-        <f>IF(N(L17)=0,"",M17/L17)</f>
+        <f>IFERROR(M17/L17,"")</f>
         <v/>
       </c>
       <c r="O17" s="12" t="inlineStr"/>
@@ -2065,7 +2069,7 @@
         <v>3.25</v>
       </c>
       <c r="N18" s="16">
-        <f>IF(N(L18)=0,"",M18/L18)</f>
+        <f>IFERROR(M18/L18,"")</f>
         <v/>
       </c>
       <c r="O18" s="12" t="inlineStr"/>
@@ -2126,7 +2130,7 @@
         <v>2.866666666666667</v>
       </c>
       <c r="N19" s="16">
-        <f>IF(N(L19)=0,"",M19/L19)</f>
+        <f>IFERROR(M19/L19,"")</f>
         <v/>
       </c>
       <c r="O19" s="12" t="inlineStr"/>
@@ -2187,7 +2191,7 @@
         <v>1.333333333333333</v>
       </c>
       <c r="N20" s="16">
-        <f>IF(N(L20)=0,"",M20/L20)</f>
+        <f>IFERROR(M20/L20,"")</f>
         <v/>
       </c>
       <c r="O20" s="12" t="inlineStr"/>
@@ -2248,7 +2252,7 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="N21" s="16">
-        <f>IF(N(L21)=0,"",M21/L21)</f>
+        <f>IFERROR(M21/L21,"")</f>
         <v/>
       </c>
       <c r="O21" s="12" t="inlineStr"/>
@@ -2309,7 +2313,7 @@
         <v>2</v>
       </c>
       <c r="N22" s="16">
-        <f>IF(N(L22)=0,"",M22/L22)</f>
+        <f>IFERROR(M22/L22,"")</f>
         <v/>
       </c>
       <c r="O22" s="12" t="inlineStr">
@@ -2374,7 +2378,7 @@
         <v>1.75</v>
       </c>
       <c r="N23" s="16">
-        <f>IF(N(L23)=0,"",M23/L23)</f>
+        <f>IFERROR(M23/L23,"")</f>
         <v/>
       </c>
       <c r="O23" s="12" t="inlineStr">
@@ -2439,7 +2443,7 @@
         <v>1.25</v>
       </c>
       <c r="N24" s="16">
-        <f>IF(N(L24)=0,"",M24/L24)</f>
+        <f>IFERROR(M24/L24,"")</f>
         <v/>
       </c>
       <c r="O24" s="12" t="inlineStr"/>
@@ -2500,7 +2504,7 @@
         <v>1</v>
       </c>
       <c r="N25" s="16">
-        <f>IF(N(L25)=0,"",M25/L25)</f>
+        <f>IFERROR(M25/L25,"")</f>
         <v/>
       </c>
       <c r="O25" s="12" t="inlineStr"/>
@@ -2561,7 +2565,7 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="N26" s="16">
-        <f>IF(N(L26)=0,"",M26/L26)</f>
+        <f>IFERROR(M26/L26,"")</f>
         <v/>
       </c>
       <c r="O26" s="12" t="inlineStr"/>
@@ -2622,7 +2626,7 @@
         <v>0</v>
       </c>
       <c r="N27" s="16">
-        <f>IF(N(L27)=0,"",M27/L27)</f>
+        <f>IFERROR(M27/L27,"")</f>
         <v/>
       </c>
       <c r="O27" s="12" t="inlineStr"/>
@@ -2679,7 +2683,7 @@
       <c r="L28" s="15" t="n"/>
       <c r="M28" s="15" t="n"/>
       <c r="N28" s="16">
-        <f>IF(N(L28)=0,"",M28/L28)</f>
+        <f>IFERROR(M28/L28,"")</f>
         <v/>
       </c>
       <c r="O28" s="12" t="inlineStr">
@@ -2736,7 +2740,7 @@
       <c r="L29" s="15" t="n"/>
       <c r="M29" s="15" t="n"/>
       <c r="N29" s="16">
-        <f>IF(N(L29)=0,"",M29/L29)</f>
+        <f>IFERROR(M29/L29,"")</f>
         <v/>
       </c>
       <c r="O29" s="12" t="inlineStr"/>
@@ -2797,7 +2801,7 @@
         <v>8.4</v>
       </c>
       <c r="N30" s="16">
-        <f>IF(N(L30)=0,"",M30/L30)</f>
+        <f>IFERROR(M30/L30,"")</f>
         <v/>
       </c>
       <c r="O30" s="12" t="inlineStr"/>
@@ -2858,7 +2862,7 @@
       <c r="L31" s="15" t="n"/>
       <c r="M31" s="15" t="n"/>
       <c r="N31" s="16">
-        <f>IF(N(L31)=0,"",M31/L31)</f>
+        <f>IFERROR(M31/L31,"")</f>
         <v/>
       </c>
       <c r="O31" s="12" t="inlineStr"/>
@@ -2923,7 +2927,7 @@
         <v>8.142857142857142</v>
       </c>
       <c r="N32" s="16">
-        <f>IF(N(L32)=0,"",M32/L32)</f>
+        <f>IFERROR(M32/L32,"")</f>
         <v/>
       </c>
       <c r="O32" s="12" t="inlineStr"/>
@@ -2984,7 +2988,7 @@
         <v>2.714285714285714</v>
       </c>
       <c r="N33" s="16">
-        <f>IF(N(L33)=0,"",M33/L33)</f>
+        <f>IFERROR(M33/L33,"")</f>
         <v/>
       </c>
       <c r="O33" s="12" t="inlineStr">
@@ -3049,7 +3053,7 @@
         <v>2.333333333333333</v>
       </c>
       <c r="N34" s="16">
-        <f>IF(N(L34)=0,"",M34/L34)</f>
+        <f>IFERROR(M34/L34,"")</f>
         <v/>
       </c>
       <c r="O34" s="12" t="inlineStr"/>
@@ -3110,7 +3114,7 @@
         <v>2.258064516129032</v>
       </c>
       <c r="N35" s="16">
-        <f>IF(N(L35)=0,"",M35/L35)</f>
+        <f>IFERROR(M35/L35,"")</f>
         <v/>
       </c>
       <c r="O35" s="12" t="inlineStr"/>
@@ -3171,7 +3175,7 @@
         <v>2</v>
       </c>
       <c r="N36" s="16">
-        <f>IF(N(L36)=0,"",M36/L36)</f>
+        <f>IFERROR(M36/L36,"")</f>
         <v/>
       </c>
       <c r="O36" s="12" t="inlineStr"/>
@@ -3232,7 +3236,7 @@
         <v>1.75</v>
       </c>
       <c r="N37" s="16">
-        <f>IF(N(L37)=0,"",M37/L37)</f>
+        <f>IFERROR(M37/L37,"")</f>
         <v/>
       </c>
       <c r="O37" s="12" t="inlineStr">
@@ -3297,7 +3301,7 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="N38" s="16">
-        <f>IF(N(L38)=0,"",M38/L38)</f>
+        <f>IFERROR(M38/L38,"")</f>
         <v/>
       </c>
       <c r="O38" s="12" t="inlineStr"/>
@@ -3358,7 +3362,7 @@
         <v>5.461538461538462</v>
       </c>
       <c r="N39" s="16">
-        <f>IF(N(L39)=0,"",M39/L39)</f>
+        <f>IFERROR(M39/L39,"")</f>
         <v/>
       </c>
       <c r="O39" s="12" t="inlineStr"/>
@@ -3419,7 +3423,7 @@
         <v>7.4</v>
       </c>
       <c r="N40" s="16">
-        <f>IF(N(L40)=0,"",M40/L40)</f>
+        <f>IFERROR(M40/L40,"")</f>
         <v/>
       </c>
       <c r="O40" s="12" t="inlineStr"/>
@@ -3484,7 +3488,7 @@
         <v>5</v>
       </c>
       <c r="N41" s="16">
-        <f>IF(N(L41)=0,"",M41/L41)</f>
+        <f>IFERROR(M41/L41,"")</f>
         <v/>
       </c>
       <c r="O41" s="12" t="inlineStr"/>
@@ -3545,7 +3549,7 @@
         <v>13.09090909090909</v>
       </c>
       <c r="N42" s="16">
-        <f>IF(N(L42)=0,"",M42/L42)</f>
+        <f>IFERROR(M42/L42,"")</f>
         <v/>
       </c>
       <c r="O42" s="12" t="inlineStr"/>
@@ -3610,7 +3614,7 @@
         <v>7.5</v>
       </c>
       <c r="N43" s="16">
-        <f>IF(N(L43)=0,"",M43/L43)</f>
+        <f>IFERROR(M43/L43,"")</f>
         <v/>
       </c>
       <c r="O43" s="12" t="inlineStr"/>
@@ -3671,7 +3675,7 @@
         <v>0</v>
       </c>
       <c r="N44" s="16">
-        <f>IF(N(L44)=0,"",M44/L44)</f>
+        <f>IFERROR(M44/L44,"")</f>
         <v/>
       </c>
       <c r="O44" s="12" t="inlineStr"/>
@@ -3732,7 +3736,7 @@
         <v>3.16</v>
       </c>
       <c r="N45" s="16">
-        <f>IF(N(L45)=0,"",M45/L45)</f>
+        <f>IFERROR(M45/L45,"")</f>
         <v/>
       </c>
       <c r="O45" s="12" t="inlineStr"/>
@@ -3793,7 +3797,7 @@
         <v>2.4</v>
       </c>
       <c r="N46" s="16">
-        <f>IF(N(L46)=0,"",M46/L46)</f>
+        <f>IFERROR(M46/L46,"")</f>
         <v/>
       </c>
       <c r="O46" s="12" t="inlineStr"/>
@@ -3854,7 +3858,7 @@
         <v>1.958333333333333</v>
       </c>
       <c r="N47" s="16">
-        <f>IF(N(L47)=0,"",M47/L47)</f>
+        <f>IFERROR(M47/L47,"")</f>
         <v/>
       </c>
       <c r="O47" s="12" t="inlineStr"/>
@@ -3915,7 +3919,7 @@
         <v>1.333333333333333</v>
       </c>
       <c r="N48" s="16">
-        <f>IF(N(L48)=0,"",M48/L48)</f>
+        <f>IFERROR(M48/L48,"")</f>
         <v/>
       </c>
       <c r="O48" s="12" t="inlineStr"/>
@@ -3976,7 +3980,7 @@
         <v>1</v>
       </c>
       <c r="N49" s="16">
-        <f>IF(N(L49)=0,"",M49/L49)</f>
+        <f>IFERROR(M49/L49,"")</f>
         <v/>
       </c>
       <c r="O49" s="12" t="inlineStr"/>
@@ -4033,7 +4037,7 @@
       <c r="L50" s="15" t="n"/>
       <c r="M50" s="15" t="n"/>
       <c r="N50" s="16">
-        <f>IF(N(L50)=0,"",M50/L50)</f>
+        <f>IFERROR(M50/L50,"")</f>
         <v/>
       </c>
       <c r="O50" s="12" t="inlineStr"/>
@@ -4094,7 +4098,7 @@
         <v>1.96551724137931</v>
       </c>
       <c r="N51" s="16">
-        <f>IF(N(L51)=0,"",M51/L51)</f>
+        <f>IFERROR(M51/L51,"")</f>
         <v/>
       </c>
       <c r="O51" s="12" t="inlineStr"/>
@@ -4155,7 +4159,7 @@
         <v>1.925</v>
       </c>
       <c r="N52" s="16">
-        <f>IF(N(L52)=0,"",M52/L52)</f>
+        <f>IFERROR(M52/L52,"")</f>
         <v/>
       </c>
       <c r="O52" s="12" t="inlineStr"/>
@@ -4216,7 +4220,7 @@
         <v>1.166666666666667</v>
       </c>
       <c r="N53" s="16">
-        <f>IF(N(L53)=0,"",M53/L53)</f>
+        <f>IFERROR(M53/L53,"")</f>
         <v/>
       </c>
       <c r="O53" s="12" t="inlineStr"/>
@@ -4277,7 +4281,7 @@
         <v>1.111111111111111</v>
       </c>
       <c r="N54" s="16">
-        <f>IF(N(L54)=0,"",M54/L54)</f>
+        <f>IFERROR(M54/L54,"")</f>
         <v/>
       </c>
       <c r="O54" s="12" t="inlineStr"/>
@@ -4338,7 +4342,7 @@
         <v>2.111111111111111</v>
       </c>
       <c r="N55" s="16">
-        <f>IF(N(L55)=0,"",M55/L55)</f>
+        <f>IFERROR(M55/L55,"")</f>
         <v/>
       </c>
       <c r="O55" s="12" t="inlineStr"/>
@@ -4399,7 +4403,7 @@
         <v>2.066666666666667</v>
       </c>
       <c r="N56" s="16">
-        <f>IF(N(L56)=0,"",M56/L56)</f>
+        <f>IFERROR(M56/L56,"")</f>
         <v/>
       </c>
       <c r="O56" s="12" t="inlineStr"/>
@@ -4460,7 +4464,7 @@
         <v>0</v>
       </c>
       <c r="N57" s="16">
-        <f>IF(N(L57)=0,"",M57/L57)</f>
+        <f>IFERROR(M57/L57,"")</f>
         <v/>
       </c>
       <c r="O57" s="12" t="inlineStr"/>
@@ -4521,7 +4525,7 @@
         <v>5</v>
       </c>
       <c r="N58" s="16">
-        <f>IF(N(L58)=0,"",M58/L58)</f>
+        <f>IFERROR(M58/L58,"")</f>
         <v/>
       </c>
       <c r="O58" s="12" t="inlineStr"/>
@@ -4582,7 +4586,7 @@
         <v>2.727272727272727</v>
       </c>
       <c r="N59" s="16">
-        <f>IF(N(L59)=0,"",M59/L59)</f>
+        <f>IFERROR(M59/L59,"")</f>
         <v/>
       </c>
       <c r="O59" s="12" t="inlineStr"/>
@@ -4643,7 +4647,7 @@
         <v>0</v>
       </c>
       <c r="N60" s="16">
-        <f>IF(N(L60)=0,"",M60/L60)</f>
+        <f>IFERROR(M60/L60,"")</f>
         <v/>
       </c>
       <c r="O60" s="12" t="inlineStr"/>
@@ -4704,7 +4708,7 @@
         <v>7</v>
       </c>
       <c r="N61" s="16">
-        <f>IF(N(L61)=0,"",M61/L61)</f>
+        <f>IFERROR(M61/L61,"")</f>
         <v/>
       </c>
       <c r="O61" s="12" t="inlineStr"/>
@@ -4769,7 +4773,7 @@
         <v>5</v>
       </c>
       <c r="N62" s="16">
-        <f>IF(N(L62)=0,"",M62/L62)</f>
+        <f>IFERROR(M62/L62,"")</f>
         <v/>
       </c>
       <c r="O62" s="12" t="inlineStr"/>
@@ -4830,7 +4834,7 @@
         <v>1.8125</v>
       </c>
       <c r="N63" s="16">
-        <f>IF(N(L63)=0,"",M63/L63)</f>
+        <f>IFERROR(M63/L63,"")</f>
         <v/>
       </c>
       <c r="O63" s="12" t="inlineStr"/>
@@ -4887,7 +4891,7 @@
       <c r="L64" s="15" t="n"/>
       <c r="M64" s="15" t="n"/>
       <c r="N64" s="16">
-        <f>IF(N(L64)=0,"",M64/L64)</f>
+        <f>IFERROR(M64/L64,"")</f>
         <v/>
       </c>
       <c r="O64" s="12" t="inlineStr"/>
@@ -4897,6 +4901,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
@@ -5288,6 +5293,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
@@ -5437,7 +5443,7 @@
         <v>3.333333333333333</v>
       </c>
       <c r="K2" s="20">
-        <f>IF(N(I2)=0,"",J2/I2)</f>
+        <f>IFERROR(J2/I2,"")</f>
         <v/>
       </c>
       <c r="L2" s="12" t="n">
@@ -5487,7 +5493,7 @@
         <v>3.75</v>
       </c>
       <c r="K3" s="20">
-        <f>IF(N(I3)=0,"",J3/I3)</f>
+        <f>IFERROR(J3/I3,"")</f>
         <v/>
       </c>
       <c r="L3" s="12" t="n">
@@ -5537,7 +5543,7 @@
         <v>4.285714285714286</v>
       </c>
       <c r="K4" s="20">
-        <f>IF(N(I4)=0,"",J4/I4)</f>
+        <f>IFERROR(J4/I4,"")</f>
         <v/>
       </c>
       <c r="L4" s="12" t="n">
@@ -5587,7 +5593,7 @@
         <v>5</v>
       </c>
       <c r="K5" s="20">
-        <f>IF(N(I5)=0,"",J5/I5)</f>
+        <f>IFERROR(J5/I5,"")</f>
         <v/>
       </c>
       <c r="L5" s="12" t="n">
@@ -5637,7 +5643,7 @@
         <v>3.833333333333333</v>
       </c>
       <c r="K6" s="20">
-        <f>IF(N(I6)=0,"",J6/I6)</f>
+        <f>IFERROR(J6/I6,"")</f>
         <v/>
       </c>
       <c r="L6" s="12" t="n">
@@ -5687,7 +5693,7 @@
         <v>6.6</v>
       </c>
       <c r="K7" s="20">
-        <f>IF(N(I7)=0,"",J7/I7)</f>
+        <f>IFERROR(J7/I7,"")</f>
         <v/>
       </c>
       <c r="L7" s="12" t="n">
@@ -5737,7 +5743,7 @@
         <v>3.25</v>
       </c>
       <c r="K8" s="20">
-        <f>IF(N(I8)=0,"",J8/I8)</f>
+        <f>IFERROR(J8/I8,"")</f>
         <v/>
       </c>
       <c r="L8" s="12" t="n">
@@ -5787,7 +5793,7 @@
         <v>6</v>
       </c>
       <c r="K9" s="20">
-        <f>IF(N(I9)=0,"",J9/I9)</f>
+        <f>IFERROR(J9/I9,"")</f>
         <v/>
       </c>
       <c r="L9" s="12" t="n">
@@ -5837,7 +5843,7 @@
         <v>5</v>
       </c>
       <c r="K10" s="20">
-        <f>IF(N(I10)=0,"",J10/I10)</f>
+        <f>IFERROR(J10/I10,"")</f>
         <v/>
       </c>
       <c r="L10" s="12" t="n">
@@ -5883,7 +5889,7 @@
       <c r="I11" s="18" t="n"/>
       <c r="J11" s="18" t="n"/>
       <c r="K11" s="20">
-        <f>IF(N(I11)=0,"",J11/I11)</f>
+        <f>IFERROR(J11/I11,"")</f>
         <v/>
       </c>
       <c r="L11" s="12" t="n">
@@ -5933,7 +5939,7 @@
         <v>9</v>
       </c>
       <c r="K12" s="20">
-        <f>IF(N(I12)=0,"",J12/I12)</f>
+        <f>IFERROR(J12/I12,"")</f>
         <v/>
       </c>
       <c r="L12" s="12" t="n">
@@ -5983,7 +5989,7 @@
         <v>2.25</v>
       </c>
       <c r="K13" s="20">
-        <f>IF(N(I13)=0,"",J13/I13)</f>
+        <f>IFERROR(J13/I13,"")</f>
         <v/>
       </c>
       <c r="L13" s="12" t="n">
@@ -6033,7 +6039,7 @@
         <v>5</v>
       </c>
       <c r="K14" s="20">
-        <f>IF(N(I14)=0,"",J14/I14)</f>
+        <f>IFERROR(J14/I14,"")</f>
         <v/>
       </c>
       <c r="L14" s="12" t="n">
@@ -6083,7 +6089,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="20">
-        <f>IF(N(I15)=0,"",J15/I15)</f>
+        <f>IFERROR(J15/I15,"")</f>
         <v/>
       </c>
       <c r="L15" s="12" t="n">
@@ -6133,7 +6139,7 @@
         <v>6</v>
       </c>
       <c r="K16" s="20">
-        <f>IF(N(I16)=0,"",J16/I16)</f>
+        <f>IFERROR(J16/I16,"")</f>
         <v/>
       </c>
       <c r="L16" s="12" t="n">
@@ -6179,7 +6185,7 @@
       <c r="I17" s="18" t="n"/>
       <c r="J17" s="18" t="n"/>
       <c r="K17" s="20">
-        <f>IF(N(I17)=0,"",J17/I17)</f>
+        <f>IFERROR(J17/I17,"")</f>
         <v/>
       </c>
       <c r="L17" s="12" t="n">
@@ -6225,7 +6231,7 @@
       <c r="I18" s="18" t="n"/>
       <c r="J18" s="18" t="n"/>
       <c r="K18" s="20">
-        <f>IF(N(I18)=0,"",J18/I18)</f>
+        <f>IFERROR(J18/I18,"")</f>
         <v/>
       </c>
       <c r="L18" s="12" t="n">
@@ -6271,7 +6277,7 @@
       <c r="I19" s="18" t="n"/>
       <c r="J19" s="18" t="n"/>
       <c r="K19" s="20">
-        <f>IF(N(I19)=0,"",J19/I19)</f>
+        <f>IFERROR(J19/I19,"")</f>
         <v/>
       </c>
       <c r="L19" s="12" t="n">
@@ -6283,6 +6289,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
@@ -6526,6 +6533,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Count sets that were played, not set slots that were recorded
Volleyball Life files a best-of-three as three slots and fills the
unplayed decider with [0, 0], so len(sets) turns every straight-sets win
into three sets. A quarter of the slots in the reference divisions the
planning page uses -- 1,347 of 5,496 -- are those placeholders, so every
sets and contested figure drawn from a Volleyball Life event was inflated
by about a third. CBVA is barely affected at 1.2%, which is why the
distortion favoured the national events over the open circuit.

Found while comparing the 17U and 18U draws at the AVP Juniors West
Coast Championships, where it made both divisions look like three sets a
match. The headline number moves with it: the biggest event on the
calendar gives 18 sets, not 24.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CyJT87Xw81b5gvhLUekjFd
</commit_message>
<xml_diff>
--- a/docs/plan-2027.xlsx
+++ b/docs/plan-2027.xlsx
@@ -645,7 +645,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Built 20 October 2026 from the Volleyball Life crawl and CBVA’s tournament database.</t>
+          <t>Built 22 October 2026 from the Volleyball Life crawl and CBVA’s tournament database.</t>
         </is>
       </c>
     </row>
@@ -1130,10 +1130,10 @@
         <v>17</v>
       </c>
       <c r="L3" s="15" t="n">
-        <v>14.66666666666667</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="M3" s="15" t="n">
-        <v>7</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="N3" s="16">
         <f>IFERROR(M3/L3,"")</f>
@@ -1195,10 +1195,10 @@
         <v>0</v>
       </c>
       <c r="L4" s="15" t="n">
-        <v>15</v>
+        <v>9.666666666666666</v>
       </c>
       <c r="M4" s="15" t="n">
-        <v>5</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="N4" s="16">
         <f>IFERROR(M4/L4,"")</f>
@@ -1840,7 +1840,7 @@
         <v>6</v>
       </c>
       <c r="L15" s="15" t="n">
-        <v>2.5</v>
+        <v>2.25</v>
       </c>
       <c r="M15" s="15" t="n">
         <v>1</v>
@@ -1962,10 +1962,10 @@
         <v>8</v>
       </c>
       <c r="L17" s="15" t="n">
-        <v>7.75</v>
+        <v>6.25</v>
       </c>
       <c r="M17" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N17" s="16">
         <f>IFERROR(M17/L17,"")</f>
@@ -2076,10 +2076,10 @@
         <v>8</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>7.75</v>
+        <v>6.25</v>
       </c>
       <c r="M19" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N19" s="16">
         <f>IFERROR(M19/L19,"")</f>
@@ -2141,10 +2141,10 @@
         <v>9</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>21</v>
+        <v>16.125</v>
       </c>
       <c r="M20" s="15" t="n">
-        <v>8.25</v>
+        <v>7</v>
       </c>
       <c r="N20" s="16">
         <f>IFERROR(M20/L20,"")</f>
@@ -2202,10 +2202,10 @@
         <v>4</v>
       </c>
       <c r="L21" s="15" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M21" s="15" t="n">
-        <v>11</v>
+        <v>9.333333333333334</v>
       </c>
       <c r="N21" s="16">
         <f>IFERROR(M21/L21,"")</f>
@@ -2267,10 +2267,10 @@
         <v>4</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>12.5</v>
+        <v>8.666666666666666</v>
       </c>
       <c r="M22" s="15" t="n">
-        <v>9.5</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="N22" s="16">
         <f>IFERROR(M22/L22,"")</f>
@@ -2393,10 +2393,10 @@
         <v>4</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M24" s="15" t="n">
-        <v>11</v>
+        <v>9.333333333333334</v>
       </c>
       <c r="N24" s="16">
         <f>IFERROR(M24/L24,"")</f>
@@ -2511,10 +2511,10 @@
         <v>17</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="M26" s="15" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="N26" s="16">
         <f>IFERROR(M26/L26,"")</f>
@@ -2572,10 +2572,10 @@
         <v>1</v>
       </c>
       <c r="L27" s="15" t="n">
-        <v>8.333333333333334</v>
+        <v>6.333333333333333</v>
       </c>
       <c r="M27" s="15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N27" s="16">
         <f>IFERROR(M27/L27,"")</f>
@@ -2696,10 +2696,10 @@
         <v>6</v>
       </c>
       <c r="L29" s="15" t="n">
-        <v>9.266666666666667</v>
+        <v>7.133333333333334</v>
       </c>
       <c r="M29" s="15" t="n">
-        <v>5.933333333333334</v>
+        <v>4.533333333333333</v>
       </c>
       <c r="N29" s="16">
         <f>IFERROR(M29/L29,"")</f>
@@ -2826,7 +2826,7 @@
         <v>2</v>
       </c>
       <c r="L31" s="15" t="n">
-        <v>5.25</v>
+        <v>4.75</v>
       </c>
       <c r="M31" s="15" t="n">
         <v>0.75</v>
@@ -3676,10 +3676,10 @@
         <v>1</v>
       </c>
       <c r="L45" s="15" t="n">
-        <v>17.4</v>
+        <v>13.2</v>
       </c>
       <c r="M45" s="15" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
       <c r="N45" s="16">
         <f>IFERROR(M45/L45,"")</f>
@@ -3802,10 +3802,10 @@
         <v>6</v>
       </c>
       <c r="L47" s="15" t="n">
-        <v>15.42857142857143</v>
+        <v>11.85714285714286</v>
       </c>
       <c r="M47" s="15" t="n">
-        <v>8.142857142857142</v>
+        <v>6.714285714285714</v>
       </c>
       <c r="N47" s="16">
         <f>IFERROR(M47/L47,"")</f>
@@ -4237,10 +4237,10 @@
         <v>14</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>17.69230769230769</v>
+        <v>13.15384615384615</v>
       </c>
       <c r="M54" s="15" t="n">
-        <v>5.461538461538462</v>
+        <v>4.384615384615385</v>
       </c>
       <c r="N54" s="16">
         <f>IFERROR(M54/L54,"")</f>
@@ -4298,10 +4298,10 @@
         <v>7</v>
       </c>
       <c r="L55" s="15" t="n">
-        <v>19.4</v>
+        <v>15</v>
       </c>
       <c r="M55" s="15" t="n">
-        <v>7.4</v>
+        <v>6.2</v>
       </c>
       <c r="N55" s="16">
         <f>IFERROR(M55/L55,"")</f>
@@ -4363,10 +4363,10 @@
         <v>0</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>19.66666666666667</v>
+        <v>14.33333333333333</v>
       </c>
       <c r="M56" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N56" s="16">
         <f>IFERROR(M56/L56,"")</f>
@@ -4424,10 +4424,10 @@
         <v>18</v>
       </c>
       <c r="L57" s="15" t="n">
-        <v>24.27272727272727</v>
+        <v>18</v>
       </c>
       <c r="M57" s="15" t="n">
-        <v>13.09090909090909</v>
+        <v>10.45454545454546</v>
       </c>
       <c r="N57" s="16">
         <f>IFERROR(M57/L57,"")</f>
@@ -4489,10 +4489,10 @@
         <v>3</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>22.5</v>
+        <v>15</v>
       </c>
       <c r="M58" s="15" t="n">
-        <v>7.5</v>
+        <v>5.25</v>
       </c>
       <c r="N58" s="16">
         <f>IFERROR(M58/L58,"")</f>
@@ -4550,7 +4550,7 @@
         <v>1</v>
       </c>
       <c r="L59" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M59" s="15" t="n">
         <v>0</v>
@@ -4611,10 +4611,10 @@
         <v>20</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>5.52</v>
+        <v>5.04</v>
       </c>
       <c r="M60" s="15" t="n">
-        <v>3.16</v>
+        <v>2.96</v>
       </c>
       <c r="N60" s="16">
         <f>IFERROR(M60/L60,"")</f>
@@ -5400,10 +5400,10 @@
         <v>27</v>
       </c>
       <c r="L73" s="15" t="n">
-        <v>11.33333333333333</v>
+        <v>9</v>
       </c>
       <c r="M73" s="15" t="n">
-        <v>5</v>
+        <v>4.111111111111111</v>
       </c>
       <c r="N73" s="16">
         <f>IFERROR(M73/L73,"")</f>
@@ -5583,10 +5583,10 @@
         <v>17</v>
       </c>
       <c r="L76" s="15" t="n">
-        <v>14.66666666666667</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="M76" s="15" t="n">
-        <v>7</v>
+        <v>5.555555555555555</v>
       </c>
       <c r="N76" s="16">
         <f>IFERROR(M76/L76,"")</f>
@@ -5648,10 +5648,10 @@
         <v>0</v>
       </c>
       <c r="L77" s="15" t="n">
-        <v>15</v>
+        <v>9.666666666666666</v>
       </c>
       <c r="M77" s="15" t="n">
-        <v>5</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="N77" s="16">
         <f>IFERROR(M77/L77,"")</f>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="I3" s="18" t="n"/>
       <c r="J3" s="18" t="n">
-        <v>11</v>
+        <v>9.333333333333334</v>
       </c>
       <c r="K3" s="18">
         <f>SUM(I3:J3)</f>
@@ -6016,10 +6016,10 @@
         <v>10</v>
       </c>
       <c r="I4" s="18" t="n">
-        <v>5.933333333333334</v>
+        <v>4.533333333333333</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K4" s="18">
         <f>SUM(I4:J4)</f>
@@ -6365,10 +6365,10 @@
         <v>17</v>
       </c>
       <c r="I2" s="18" t="n">
-        <v>6.166666666666667</v>
+        <v>5.333333333333333</v>
       </c>
       <c r="J2" s="18" t="n">
-        <v>3.333333333333333</v>
+        <v>3</v>
       </c>
       <c r="K2" s="20">
         <f>IFERROR(J2/I2,"")</f>
@@ -6415,10 +6415,10 @@
         <v>18</v>
       </c>
       <c r="I3" s="18" t="n">
-        <v>10</v>
+        <v>8.75</v>
       </c>
       <c r="J3" s="18" t="n">
-        <v>3.75</v>
+        <v>3.25</v>
       </c>
       <c r="K3" s="20">
         <f>IFERROR(J3/I3,"")</f>
@@ -6465,10 +6465,10 @@
         <v>16</v>
       </c>
       <c r="I4" s="18" t="n">
-        <v>9.857142857142858</v>
+        <v>7</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>4.285714285714286</v>
+        <v>2.857142857142857</v>
       </c>
       <c r="K4" s="20">
         <f>IFERROR(J4/I4,"")</f>
@@ -6515,10 +6515,10 @@
         <v>27</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>11.33333333333333</v>
+        <v>9</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>5</v>
+        <v>4.111111111111111</v>
       </c>
       <c r="K5" s="20">
         <f>IFERROR(J5/I5,"")</f>
@@ -6565,10 +6565,10 @@
         <v>18</v>
       </c>
       <c r="I6" s="18" t="n">
-        <v>7.166666666666667</v>
+        <v>6.166666666666667</v>
       </c>
       <c r="J6" s="18" t="n">
-        <v>3.833333333333333</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="K6" s="20">
         <f>IFERROR(J6/I6,"")</f>
@@ -6615,10 +6615,10 @@
         <v>13</v>
       </c>
       <c r="I7" s="18" t="n">
-        <v>12</v>
+        <v>10.2</v>
       </c>
       <c r="J7" s="18" t="n">
-        <v>6.6</v>
+        <v>5.8</v>
       </c>
       <c r="K7" s="20">
         <f>IFERROR(J7/I7,"")</f>
@@ -6665,10 +6665,10 @@
         <v>17</v>
       </c>
       <c r="I8" s="18" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="J8" s="18" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="K8" s="20">
         <f>IFERROR(J8/I8,"")</f>
@@ -6715,10 +6715,10 @@
         <v>10</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>11.4</v>
+        <v>8.6</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K9" s="20">
         <f>IFERROR(J9/I9,"")</f>
@@ -6765,10 +6765,10 @@
         <v>7</v>
       </c>
       <c r="I10" s="18" t="n">
-        <v>10.33333333333333</v>
+        <v>7.333333333333333</v>
       </c>
       <c r="J10" s="18" t="n">
-        <v>5</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="K10" s="20">
         <f>IFERROR(J10/I10,"")</f>
@@ -6861,10 +6861,10 @@
         <v>2</v>
       </c>
       <c r="I12" s="18" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J12" s="18" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K12" s="20">
         <f>IFERROR(J12/I12,"")</f>
@@ -6911,7 +6911,7 @@
         <v>14</v>
       </c>
       <c r="I13" s="18" t="n">
-        <v>5.5</v>
+        <v>4.75</v>
       </c>
       <c r="J13" s="18" t="n">
         <v>2.25</v>
@@ -6961,7 +6961,7 @@
         <v>5</v>
       </c>
       <c r="I14" s="18" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J14" s="18" t="n">
         <v>5</v>
@@ -7011,7 +7011,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J15" s="18" t="n">
         <v>0</v>
@@ -7061,10 +7061,10 @@
         <v>16</v>
       </c>
       <c r="I16" s="18" t="n">
-        <v>8.800000000000001</v>
+        <v>7.2</v>
       </c>
       <c r="J16" s="18" t="n">
-        <v>6</v>
+        <v>5.2</v>
       </c>
       <c r="K16" s="20">
         <f>IFERROR(J16/I16,"")</f>

</xml_diff>